<commit_message>
Track of the data for movements: goods receipt, issue oder tranfer. Save/Load optional
</commit_message>
<xml_diff>
--- a/ProjectSemester/warehouse_data.xlsx
+++ b/ProjectSemester/warehouse_data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="38">
   <si>
     <t>Material ID</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>Back-up material</t>
+  </si>
+  <si>
+    <t>Material to dispose</t>
   </si>
   <si>
     <t>Product ID</t>
@@ -552,7 +555,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -577,6 +580,14 @@
       </c>
       <c r="B3" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -590,7 +601,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -601,24 +612,24 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -632,18 +643,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -654,7 +665,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -665,7 +676,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -676,7 +687,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -691,7 +702,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -702,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -713,18 +724,51 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>95</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C3">
-        <v>25</v>
+      <c r="C5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>